<commit_message>
Implemente feature selection en select_data.py segun lo que habia hecho caro. Aun no esta terminado pero es un avance grande.
</commit_message>
<xml_diff>
--- a/modeling/data/df_modelos.xlsx
+++ b/modeling/data/df_modelos.xlsx
@@ -455,10 +455,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>57.6</v>
+        <v>51.98688524590165</v>
       </c>
       <c r="D2" t="n">
-        <v>75.148</v>
+        <v>53.959868852459</v>
       </c>
     </row>
     <row r="3">
@@ -471,10 +471,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>60.8</v>
+        <v>60.24918032786886</v>
       </c>
       <c r="D3" t="n">
-        <v>73.51199999999999</v>
+        <v>71.47265573770476</v>
       </c>
     </row>
     <row r="4">
@@ -497,10 +497,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>58.8</v>
+        <v>59.47540983606557</v>
       </c>
       <c r="D4" t="n">
-        <v>77.864</v>
+        <v>70.76262295081952</v>
       </c>
     </row>
     <row r="5">
@@ -513,10 +513,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>41.2</v>
+        <v>35.69836065573772</v>
       </c>
       <c r="D5" t="n">
-        <v>15.364</v>
+        <v>8.342557377049165</v>
       </c>
     </row>
     <row r="6">
@@ -529,10 +529,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>44</v>
+        <v>37.27213114754098</v>
       </c>
       <c r="D6" t="n">
-        <v>30.13600000000001</v>
+        <v>7.433704918032812</v>
       </c>
     </row>
     <row r="7">
@@ -546,10 +546,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>44.8</v>
+        <v>35.72459016393443</v>
       </c>
       <c r="D7" t="n">
-        <v>25.27599999999999</v>
+        <v>1.799213114754143</v>
       </c>
     </row>
     <row r="8">
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>62</v>
+        <v>56.95737704918033</v>
       </c>
       <c r="D8" t="n">
-        <v>81.66800000000001</v>
+        <v>63.53626229508184</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Me di cuenta de lo importante que es hacer el fillna() despues de eliminar las variables mas correlacionadas y de seleccionar las variables mas importantes. Por ello hago el clean data despues.
Consegui una precision del 95% y un roi de 170% haciendo la seleccion de variables mas importantes y eliminando las correlacionadas (antes obtenia un 65% de prec y un roi de hasta 70%)
</commit_message>
<xml_diff>
--- a/modeling/data/df_modelos.xlsx
+++ b/modeling/data/df_modelos.xlsx
@@ -455,10 +455,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>51.98688524590165</v>
+        <v>94.15081967213114</v>
       </c>
       <c r="D2" t="n">
-        <v>53.959868852459</v>
+        <v>170.7131168114542</v>
       </c>
     </row>
     <row r="3">
@@ -471,10 +471,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>60.24918032786886</v>
+        <v>94.93770491803279</v>
       </c>
       <c r="D3" t="n">
-        <v>71.47265573770476</v>
+        <v>172.2570235778378</v>
       </c>
     </row>
     <row r="4">
@@ -497,10 +497,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>59.47540983606557</v>
+        <v>95.22622950819672</v>
       </c>
       <c r="D4" t="n">
-        <v>70.76262295081952</v>
+        <v>173.2023729671723</v>
       </c>
     </row>
     <row r="5">
@@ -513,10 +513,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>35.69836065573772</v>
+        <v>74.93770491803279</v>
       </c>
       <c r="D5" t="n">
-        <v>8.342557377049165</v>
+        <v>106.8678423616269</v>
       </c>
     </row>
     <row r="6">
@@ -529,10 +529,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>37.27213114754098</v>
+        <v>82.75409836065575</v>
       </c>
       <c r="D6" t="n">
-        <v>7.433704918032812</v>
+        <v>133.0824373123123</v>
       </c>
     </row>
     <row r="7">
@@ -546,10 +546,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>35.72459016393443</v>
+        <v>92.0655737704918</v>
       </c>
       <c r="D7" t="n">
-        <v>1.799213114754143</v>
+        <v>164.2101280778575</v>
       </c>
     </row>
     <row r="8">
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>56.95737704918033</v>
+        <v>95.48852459016393</v>
       </c>
       <c r="D8" t="n">
-        <v>63.53626229508184</v>
+        <v>173.8364334139034</v>
       </c>
     </row>
   </sheetData>

</xml_diff>